<commit_message>
Fix Excel sample: blank day-of-week until a date is entered
Empty Datum cell made =TEXT(A,"DDDD") read serial 0 and show "sobota" on
every row. Guard with IF(A="","",TEXT(A,"dddd")) so the day column stays
empty until the user types a date.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/vzorec-evidenca-delovnega-casa.xlsx
+++ b/public/vzorec-evidenca-delovnega-casa.xlsx
@@ -482,7 +482,7 @@
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="str">
-        <f>TEXT(A2,"DDDD")</f>
+        <f>IF(A2="","",TEXT(A2,"dddd"))</f>
         <v/>
       </c>
       <c r="C2" s="4"/>
@@ -496,7 +496,7 @@
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B3" t="str">
-        <f>TEXT(A3,"DDDD")</f>
+        <f>IF(A3="","",TEXT(A3,"dddd"))</f>
         <v/>
       </c>
       <c r="C3" s="7"/>
@@ -510,7 +510,7 @@
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
       <c r="B4" s="3" t="str">
-        <f>TEXT(A4,"DDDD")</f>
+        <f>IF(A4="","",TEXT(A4,"dddd"))</f>
         <v/>
       </c>
       <c r="C4" s="4"/>
@@ -524,7 +524,7 @@
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" t="str">
-        <f>TEXT(A5,"DDDD")</f>
+        <f>IF(A5="","",TEXT(A5,"dddd"))</f>
         <v/>
       </c>
       <c r="C5" s="7"/>
@@ -538,7 +538,7 @@
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
       <c r="B6" s="3" t="str">
-        <f>TEXT(A6,"DDDD")</f>
+        <f>IF(A6="","",TEXT(A6,"dddd"))</f>
         <v/>
       </c>
       <c r="C6" s="4"/>
@@ -552,7 +552,7 @@
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" t="str">
-        <f>TEXT(A7,"DDDD")</f>
+        <f>IF(A7="","",TEXT(A7,"dddd"))</f>
         <v/>
       </c>
       <c r="C7" s="7"/>
@@ -566,7 +566,7 @@
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
       <c r="B8" s="3" t="str">
-        <f>TEXT(A8,"DDDD")</f>
+        <f>IF(A8="","",TEXT(A8,"dddd"))</f>
         <v/>
       </c>
       <c r="C8" s="4"/>
@@ -580,7 +580,7 @@
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" t="str">
-        <f>TEXT(A9,"DDDD")</f>
+        <f>IF(A9="","",TEXT(A9,"dddd"))</f>
         <v/>
       </c>
       <c r="C9" s="7"/>
@@ -594,7 +594,7 @@
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" s="3" t="str">
-        <f>TEXT(A10,"DDDD")</f>
+        <f>IF(A10="","",TEXT(A10,"dddd"))</f>
         <v/>
       </c>
       <c r="C10" s="4"/>
@@ -608,7 +608,7 @@
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" t="str">
-        <f>TEXT(A11,"DDDD")</f>
+        <f>IF(A11="","",TEXT(A11,"dddd"))</f>
         <v/>
       </c>
       <c r="C11" s="7"/>
@@ -622,7 +622,7 @@
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" s="3" t="str">
-        <f>TEXT(A12,"DDDD")</f>
+        <f>IF(A12="","",TEXT(A12,"dddd"))</f>
         <v/>
       </c>
       <c r="C12" s="4"/>
@@ -636,7 +636,7 @@
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" t="str">
-        <f>TEXT(A13,"DDDD")</f>
+        <f>IF(A13="","",TEXT(A13,"dddd"))</f>
         <v/>
       </c>
       <c r="C13" s="7"/>
@@ -650,7 +650,7 @@
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="3" t="str">
-        <f>TEXT(A14,"DDDD")</f>
+        <f>IF(A14="","",TEXT(A14,"dddd"))</f>
         <v/>
       </c>
       <c r="C14" s="4"/>
@@ -664,7 +664,7 @@
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" t="str">
-        <f>TEXT(A15,"DDDD")</f>
+        <f>IF(A15="","",TEXT(A15,"dddd"))</f>
         <v/>
       </c>
       <c r="C15" s="7"/>
@@ -678,7 +678,7 @@
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="3" t="str">
-        <f>TEXT(A16,"DDDD")</f>
+        <f>IF(A16="","",TEXT(A16,"dddd"))</f>
         <v/>
       </c>
       <c r="C16" s="4"/>
@@ -692,7 +692,7 @@
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" t="str">
-        <f>TEXT(A17,"DDDD")</f>
+        <f>IF(A17="","",TEXT(A17,"dddd"))</f>
         <v/>
       </c>
       <c r="C17" s="7"/>
@@ -706,7 +706,7 @@
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
       <c r="B18" s="3" t="str">
-        <f>TEXT(A18,"DDDD")</f>
+        <f>IF(A18="","",TEXT(A18,"dddd"))</f>
         <v/>
       </c>
       <c r="C18" s="4"/>
@@ -720,7 +720,7 @@
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" t="str">
-        <f>TEXT(A19,"DDDD")</f>
+        <f>IF(A19="","",TEXT(A19,"dddd"))</f>
         <v/>
       </c>
       <c r="C19" s="7"/>
@@ -734,7 +734,7 @@
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="3" t="str">
-        <f>TEXT(A20,"DDDD")</f>
+        <f>IF(A20="","",TEXT(A20,"dddd"))</f>
         <v/>
       </c>
       <c r="C20" s="4"/>
@@ -748,7 +748,7 @@
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" t="str">
-        <f>TEXT(A21,"DDDD")</f>
+        <f>IF(A21="","",TEXT(A21,"dddd"))</f>
         <v/>
       </c>
       <c r="C21" s="7"/>
@@ -762,7 +762,7 @@
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
       <c r="B22" s="3" t="str">
-        <f>TEXT(A22,"DDDD")</f>
+        <f>IF(A22="","",TEXT(A22,"dddd"))</f>
         <v/>
       </c>
       <c r="C22" s="4"/>
@@ -776,7 +776,7 @@
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" t="str">
-        <f>TEXT(A23,"DDDD")</f>
+        <f>IF(A23="","",TEXT(A23,"dddd"))</f>
         <v/>
       </c>
       <c r="C23" s="7"/>
@@ -790,7 +790,7 @@
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" s="3" t="str">
-        <f>TEXT(A24,"DDDD")</f>
+        <f>IF(A24="","",TEXT(A24,"dddd"))</f>
         <v/>
       </c>
       <c r="C24" s="4"/>
@@ -804,7 +804,7 @@
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" t="str">
-        <f>TEXT(A25,"DDDD")</f>
+        <f>IF(A25="","",TEXT(A25,"dddd"))</f>
         <v/>
       </c>
       <c r="C25" s="7"/>
@@ -818,7 +818,7 @@
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
       <c r="B26" s="3" t="str">
-        <f>TEXT(A26,"DDDD")</f>
+        <f>IF(A26="","",TEXT(A26,"dddd"))</f>
         <v/>
       </c>
       <c r="C26" s="4"/>
@@ -832,7 +832,7 @@
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" t="str">
-        <f>TEXT(A27,"DDDD")</f>
+        <f>IF(A27="","",TEXT(A27,"dddd"))</f>
         <v/>
       </c>
       <c r="C27" s="7"/>
@@ -846,7 +846,7 @@
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="B28" s="3" t="str">
-        <f>TEXT(A28,"DDDD")</f>
+        <f>IF(A28="","",TEXT(A28,"dddd"))</f>
         <v/>
       </c>
       <c r="C28" s="4"/>
@@ -860,7 +860,7 @@
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29" t="str">
-        <f>TEXT(A29,"DDDD")</f>
+        <f>IF(A29="","",TEXT(A29,"dddd"))</f>
         <v/>
       </c>
       <c r="C29" s="7"/>
@@ -874,7 +874,7 @@
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="str">
-        <f>TEXT(A30,"DDDD")</f>
+        <f>IF(A30="","",TEXT(A30,"dddd"))</f>
         <v/>
       </c>
       <c r="C30" s="4"/>
@@ -888,7 +888,7 @@
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B31" t="str">
-        <f>TEXT(A31,"DDDD")</f>
+        <f>IF(A31="","",TEXT(A31,"dddd"))</f>
         <v/>
       </c>
       <c r="C31" s="7"/>
@@ -902,7 +902,7 @@
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="str">
-        <f>TEXT(A32,"DDDD")</f>
+        <f>IF(A32="","",TEXT(A32,"dddd"))</f>
         <v/>
       </c>
       <c r="C32" s="4"/>
@@ -916,7 +916,7 @@
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B33" t="str">
-        <f>TEXT(A33,"DDDD")</f>
+        <f>IF(A33="","",TEXT(A33,"dddd"))</f>
         <v/>
       </c>
       <c r="C33" s="7"/>
@@ -931,9 +931,9 @@
       <c r="A35" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="F35" s="11" t="str">
+      <c r="F35" s="11">
         <f>SUM(F2:F33)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix Excel sample day column: use WEEKDAY+CHOOSE (text), not TEXT format
TEXT(A,"dddd") could render as the date again depending on the cell's
number format. Replace with IF(A="","",CHOOSE(WEEKDAY(A,2),"ponedeljek"...))
and set the day column to text format (@) so it always shows the Slovenian
weekday name and never a date. Datum column formatted dd.mm.yyyy.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/vzorec-evidenca-delovnega-casa.xlsx
+++ b/public/vzorec-evidenca-delovnega-casa.xlsx
@@ -41,8 +41,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="hh:mm"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="dd.mm.yyyy"/>
+    <numFmt numFmtId="165" formatCode="hh:mm"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -91,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -99,11 +100,15 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="4" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -481,457 +486,473 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
-      <c r="B2" s="3" t="str">
-        <f>IF(A2="","",TEXT(A2,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="6" t="str">
+      <c r="B2" s="4" t="str">
+        <f>IF(A2="","",CHOOSE(WEEKDAY(A2,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="7" t="str">
         <f>IF(AND(C2&lt;&gt;"",D2&lt;&gt;""),(D2-C2)*24-E2/60,"")</f>
         <v/>
       </c>
-      <c r="G2" s="3"/>
-    </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B3" t="str">
-        <f>IF(A3="","",TEXT(A3,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="9" t="str">
+      <c r="G2" s="8"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="9"/>
+      <c r="B3" s="10" t="str">
+        <f>IF(A3="","",CHOOSE(WEEKDAY(A3,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="13" t="str">
         <f>IF(AND(C3&lt;&gt;"",D3&lt;&gt;""),(D3-C3)*24-E3/60,"")</f>
         <v/>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
-      <c r="B4" s="3" t="str">
-        <f>IF(A4="","",TEXT(A4,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="6" t="str">
+      <c r="B4" s="4" t="str">
+        <f>IF(A4="","",CHOOSE(WEEKDAY(A4,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="7" t="str">
         <f>IF(AND(C4&lt;&gt;"",D4&lt;&gt;""),(D4-C4)*24-E4/60,"")</f>
         <v/>
       </c>
-      <c r="G4" s="3"/>
-    </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" t="str">
-        <f>IF(A5="","",TEXT(A5,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="9" t="str">
+      <c r="G4" s="8"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="9"/>
+      <c r="B5" s="10" t="str">
+        <f>IF(A5="","",CHOOSE(WEEKDAY(A5,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="13" t="str">
         <f>IF(AND(C5&lt;&gt;"",D5&lt;&gt;""),(D5-C5)*24-E5/60,"")</f>
         <v/>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
-      <c r="B6" s="3" t="str">
-        <f>IF(A6="","",TEXT(A6,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="6" t="str">
+      <c r="B6" s="4" t="str">
+        <f>IF(A6="","",CHOOSE(WEEKDAY(A6,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="7" t="str">
         <f>IF(AND(C6&lt;&gt;"",D6&lt;&gt;""),(D6-C6)*24-E6/60,"")</f>
         <v/>
       </c>
-      <c r="G6" s="3"/>
-    </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7" t="str">
-        <f>IF(A7="","",TEXT(A7,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="9" t="str">
+      <c r="G6" s="8"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="9"/>
+      <c r="B7" s="10" t="str">
+        <f>IF(A7="","",CHOOSE(WEEKDAY(A7,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="13" t="str">
         <f>IF(AND(C7&lt;&gt;"",D7&lt;&gt;""),(D7-C7)*24-E7/60,"")</f>
         <v/>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
-      <c r="B8" s="3" t="str">
-        <f>IF(A8="","",TEXT(A8,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="6" t="str">
+      <c r="B8" s="4" t="str">
+        <f>IF(A8="","",CHOOSE(WEEKDAY(A8,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="7" t="str">
         <f>IF(AND(C8&lt;&gt;"",D8&lt;&gt;""),(D8-C8)*24-E8/60,"")</f>
         <v/>
       </c>
-      <c r="G8" s="3"/>
-    </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" t="str">
-        <f>IF(A9="","",TEXT(A9,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="9" t="str">
+      <c r="G8" s="8"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="9"/>
+      <c r="B9" s="10" t="str">
+        <f>IF(A9="","",CHOOSE(WEEKDAY(A9,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="13" t="str">
         <f>IF(AND(C9&lt;&gt;"",D9&lt;&gt;""),(D9-C9)*24-E9/60,"")</f>
         <v/>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
-      <c r="B10" s="3" t="str">
-        <f>IF(A10="","",TEXT(A10,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="6" t="str">
+      <c r="B10" s="4" t="str">
+        <f>IF(A10="","",CHOOSE(WEEKDAY(A10,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="7" t="str">
         <f>IF(AND(C10&lt;&gt;"",D10&lt;&gt;""),(D10-C10)*24-E10/60,"")</f>
         <v/>
       </c>
-      <c r="G10" s="3"/>
-    </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B11" t="str">
-        <f>IF(A11="","",TEXT(A11,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="9" t="str">
+      <c r="G10" s="8"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="9"/>
+      <c r="B11" s="10" t="str">
+        <f>IF(A11="","",CHOOSE(WEEKDAY(A11,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="13" t="str">
         <f>IF(AND(C11&lt;&gt;"",D11&lt;&gt;""),(D11-C11)*24-E11/60,"")</f>
         <v/>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
-      <c r="B12" s="3" t="str">
-        <f>IF(A12="","",TEXT(A12,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="6" t="str">
+      <c r="B12" s="4" t="str">
+        <f>IF(A12="","",CHOOSE(WEEKDAY(A12,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="7" t="str">
         <f>IF(AND(C12&lt;&gt;"",D12&lt;&gt;""),(D12-C12)*24-E12/60,"")</f>
         <v/>
       </c>
-      <c r="G12" s="3"/>
-    </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B13" t="str">
-        <f>IF(A13="","",TEXT(A13,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="9" t="str">
+      <c r="G12" s="8"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="9"/>
+      <c r="B13" s="10" t="str">
+        <f>IF(A13="","",CHOOSE(WEEKDAY(A13,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="13" t="str">
         <f>IF(AND(C13&lt;&gt;"",D13&lt;&gt;""),(D13-C13)*24-E13/60,"")</f>
         <v/>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
-      <c r="B14" s="3" t="str">
-        <f>IF(A14="","",TEXT(A14,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="6" t="str">
+      <c r="B14" s="4" t="str">
+        <f>IF(A14="","",CHOOSE(WEEKDAY(A14,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="7" t="str">
         <f>IF(AND(C14&lt;&gt;"",D14&lt;&gt;""),(D14-C14)*24-E14/60,"")</f>
         <v/>
       </c>
-      <c r="G14" s="3"/>
-    </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B15" t="str">
-        <f>IF(A15="","",TEXT(A15,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="9" t="str">
+      <c r="G14" s="8"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="9"/>
+      <c r="B15" s="10" t="str">
+        <f>IF(A15="","",CHOOSE(WEEKDAY(A15,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="13" t="str">
         <f>IF(AND(C15&lt;&gt;"",D15&lt;&gt;""),(D15-C15)*24-E15/60,"")</f>
         <v/>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
-      <c r="B16" s="3" t="str">
-        <f>IF(A16="","",TEXT(A16,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="6" t="str">
+      <c r="B16" s="4" t="str">
+        <f>IF(A16="","",CHOOSE(WEEKDAY(A16,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="7" t="str">
         <f>IF(AND(C16&lt;&gt;"",D16&lt;&gt;""),(D16-C16)*24-E16/60,"")</f>
         <v/>
       </c>
-      <c r="G16" s="3"/>
-    </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B17" t="str">
-        <f>IF(A17="","",TEXT(A17,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="9" t="str">
+      <c r="G16" s="8"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="9"/>
+      <c r="B17" s="10" t="str">
+        <f>IF(A17="","",CHOOSE(WEEKDAY(A17,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="13" t="str">
         <f>IF(AND(C17&lt;&gt;"",D17&lt;&gt;""),(D17-C17)*24-E17/60,"")</f>
         <v/>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
-      <c r="B18" s="3" t="str">
-        <f>IF(A18="","",TEXT(A18,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="6" t="str">
+      <c r="B18" s="4" t="str">
+        <f>IF(A18="","",CHOOSE(WEEKDAY(A18,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="7" t="str">
         <f>IF(AND(C18&lt;&gt;"",D18&lt;&gt;""),(D18-C18)*24-E18/60,"")</f>
         <v/>
       </c>
-      <c r="G18" s="3"/>
-    </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B19" t="str">
-        <f>IF(A19="","",TEXT(A19,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="9" t="str">
+      <c r="G18" s="8"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="9"/>
+      <c r="B19" s="10" t="str">
+        <f>IF(A19="","",CHOOSE(WEEKDAY(A19,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="13" t="str">
         <f>IF(AND(C19&lt;&gt;"",D19&lt;&gt;""),(D19-C19)*24-E19/60,"")</f>
         <v/>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
-      <c r="B20" s="3" t="str">
-        <f>IF(A20="","",TEXT(A20,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="6" t="str">
+      <c r="B20" s="4" t="str">
+        <f>IF(A20="","",CHOOSE(WEEKDAY(A20,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="7" t="str">
         <f>IF(AND(C20&lt;&gt;"",D20&lt;&gt;""),(D20-C20)*24-E20/60,"")</f>
         <v/>
       </c>
-      <c r="G20" s="3"/>
-    </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B21" t="str">
-        <f>IF(A21="","",TEXT(A21,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="9" t="str">
+      <c r="G20" s="8"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="9"/>
+      <c r="B21" s="10" t="str">
+        <f>IF(A21="","",CHOOSE(WEEKDAY(A21,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="13" t="str">
         <f>IF(AND(C21&lt;&gt;"",D21&lt;&gt;""),(D21-C21)*24-E21/60,"")</f>
         <v/>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
-      <c r="B22" s="3" t="str">
-        <f>IF(A22="","",TEXT(A22,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="6" t="str">
+      <c r="B22" s="4" t="str">
+        <f>IF(A22="","",CHOOSE(WEEKDAY(A22,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="7" t="str">
         <f>IF(AND(C22&lt;&gt;"",D22&lt;&gt;""),(D22-C22)*24-E22/60,"")</f>
         <v/>
       </c>
-      <c r="G22" s="3"/>
-    </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B23" t="str">
-        <f>IF(A23="","",TEXT(A23,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="9" t="str">
+      <c r="G22" s="8"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="9"/>
+      <c r="B23" s="10" t="str">
+        <f>IF(A23="","",CHOOSE(WEEKDAY(A23,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="13" t="str">
         <f>IF(AND(C23&lt;&gt;"",D23&lt;&gt;""),(D23-C23)*24-E23/60,"")</f>
         <v/>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
-      <c r="B24" s="3" t="str">
-        <f>IF(A24="","",TEXT(A24,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="6" t="str">
+      <c r="B24" s="4" t="str">
+        <f>IF(A24="","",CHOOSE(WEEKDAY(A24,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="7" t="str">
         <f>IF(AND(C24&lt;&gt;"",D24&lt;&gt;""),(D24-C24)*24-E24/60,"")</f>
         <v/>
       </c>
-      <c r="G24" s="3"/>
-    </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B25" t="str">
-        <f>IF(A25="","",TEXT(A25,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="9" t="str">
+      <c r="G24" s="8"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="9"/>
+      <c r="B25" s="10" t="str">
+        <f>IF(A25="","",CHOOSE(WEEKDAY(A25,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="13" t="str">
         <f>IF(AND(C25&lt;&gt;"",D25&lt;&gt;""),(D25-C25)*24-E25/60,"")</f>
         <v/>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
-      <c r="B26" s="3" t="str">
-        <f>IF(A26="","",TEXT(A26,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="6" t="str">
+      <c r="B26" s="4" t="str">
+        <f>IF(A26="","",CHOOSE(WEEKDAY(A26,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C26" s="5"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="7" t="str">
         <f>IF(AND(C26&lt;&gt;"",D26&lt;&gt;""),(D26-C26)*24-E26/60,"")</f>
         <v/>
       </c>
-      <c r="G26" s="3"/>
-    </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B27" t="str">
-        <f>IF(A27="","",TEXT(A27,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C27" s="7"/>
-      <c r="D27" s="7"/>
-      <c r="E27" s="8"/>
-      <c r="F27" s="9" t="str">
+      <c r="G26" s="8"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="9"/>
+      <c r="B27" s="10" t="str">
+        <f>IF(A27="","",CHOOSE(WEEKDAY(A27,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="13" t="str">
         <f>IF(AND(C27&lt;&gt;"",D27&lt;&gt;""),(D27-C27)*24-E27/60,"")</f>
         <v/>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
-      <c r="B28" s="3" t="str">
-        <f>IF(A28="","",TEXT(A28,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="5"/>
-      <c r="F28" s="6" t="str">
+      <c r="B28" s="4" t="str">
+        <f>IF(A28="","",CHOOSE(WEEKDAY(A28,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="6"/>
+      <c r="F28" s="7" t="str">
         <f>IF(AND(C28&lt;&gt;"",D28&lt;&gt;""),(D28-C28)*24-E28/60,"")</f>
         <v/>
       </c>
-      <c r="G28" s="3"/>
-    </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B29" t="str">
-        <f>IF(A29="","",TEXT(A29,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C29" s="7"/>
-      <c r="D29" s="7"/>
-      <c r="E29" s="8"/>
-      <c r="F29" s="9" t="str">
+      <c r="G28" s="8"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="9"/>
+      <c r="B29" s="10" t="str">
+        <f>IF(A29="","",CHOOSE(WEEKDAY(A29,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C29" s="11"/>
+      <c r="D29" s="11"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="13" t="str">
         <f>IF(AND(C29&lt;&gt;"",D29&lt;&gt;""),(D29-C29)*24-E29/60,"")</f>
         <v/>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
-      <c r="B30" s="3" t="str">
-        <f>IF(A30="","",TEXT(A30,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4"/>
-      <c r="E30" s="5"/>
-      <c r="F30" s="6" t="str">
+      <c r="B30" s="4" t="str">
+        <f>IF(A30="","",CHOOSE(WEEKDAY(A30,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C30" s="5"/>
+      <c r="D30" s="5"/>
+      <c r="E30" s="6"/>
+      <c r="F30" s="7" t="str">
         <f>IF(AND(C30&lt;&gt;"",D30&lt;&gt;""),(D30-C30)*24-E30/60,"")</f>
         <v/>
       </c>
-      <c r="G30" s="3"/>
-    </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B31" t="str">
-        <f>IF(A31="","",TEXT(A31,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C31" s="7"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="8"/>
-      <c r="F31" s="9" t="str">
+      <c r="G30" s="8"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="9"/>
+      <c r="B31" s="10" t="str">
+        <f>IF(A31="","",CHOOSE(WEEKDAY(A31,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C31" s="11"/>
+      <c r="D31" s="11"/>
+      <c r="E31" s="12"/>
+      <c r="F31" s="13" t="str">
         <f>IF(AND(C31&lt;&gt;"",D31&lt;&gt;""),(D31-C31)*24-E31/60,"")</f>
         <v/>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
-      <c r="B32" s="3" t="str">
-        <f>IF(A32="","",TEXT(A32,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C32" s="4"/>
-      <c r="D32" s="4"/>
-      <c r="E32" s="5"/>
-      <c r="F32" s="6" t="str">
+      <c r="B32" s="4" t="str">
+        <f>IF(A32="","",CHOOSE(WEEKDAY(A32,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C32" s="5"/>
+      <c r="D32" s="5"/>
+      <c r="E32" s="6"/>
+      <c r="F32" s="7" t="str">
         <f>IF(AND(C32&lt;&gt;"",D32&lt;&gt;""),(D32-C32)*24-E32/60,"")</f>
         <v/>
       </c>
-      <c r="G32" s="3"/>
-    </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B33" t="str">
-        <f>IF(A33="","",TEXT(A33,"dddd"))</f>
-        <v/>
-      </c>
-      <c r="C33" s="7"/>
-      <c r="D33" s="7"/>
-      <c r="E33" s="8"/>
-      <c r="F33" s="9" t="str">
+      <c r="G32" s="8"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="9"/>
+      <c r="B33" s="10" t="str">
+        <f>IF(A33="","",CHOOSE(WEEKDAY(A33,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <v/>
+      </c>
+      <c r="C33" s="11"/>
+      <c r="D33" s="11"/>
+      <c r="E33" s="12"/>
+      <c r="F33" s="13" t="str">
         <f>IF(AND(C33&lt;&gt;"",D33&lt;&gt;""),(D33-C33)*24-E33/60,"")</f>
         <v/>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="10" t="s">
+      <c r="A35" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="F35" s="11">
+      <c r="F35" s="15">
         <f>SUM(F2:F33)</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Excel sample: capitalize weekday names + Excel-safe day formula
- Day names now capitalized (Petek, not petek) for a more professional look.
- Wrap day formula in IFERROR and accept text dates via DATEVALUE so Excel
  shows a blank instead of #VALUE! when a typed date is stored as text
  (Google Sheets already parsed it as a real date).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/vzorec-evidenca-delovnega-casa.xlsx
+++ b/public/vzorec-evidenca-delovnega-casa.xlsx
@@ -92,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -101,13 +101,11 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="4" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -487,7 +485,7 @@
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="4" t="str">
-        <f>IF(A2="","",CHOOSE(WEEKDAY(A2,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <f>IF(A2="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A2),A2,DATEVALUE(A2)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
         <v/>
       </c>
       <c r="C2" s="5"/>
@@ -497,18 +495,18 @@
         <f>IF(AND(C2&lt;&gt;"",D2&lt;&gt;""),(D2-C2)*24-E2/60,"")</f>
         <v/>
       </c>
-      <c r="G2" s="8"/>
+      <c r="G2" s="4"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="9"/>
-      <c r="B3" s="10" t="str">
-        <f>IF(A3="","",CHOOSE(WEEKDAY(A3,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
-        <v/>
-      </c>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="13" t="str">
+      <c r="A3" s="8"/>
+      <c r="B3" t="str">
+        <f>IF(A3="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A3),A3,DATEVALUE(A3)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
+        <v/>
+      </c>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="11" t="str">
         <f>IF(AND(C3&lt;&gt;"",D3&lt;&gt;""),(D3-C3)*24-E3/60,"")</f>
         <v/>
       </c>
@@ -516,7 +514,7 @@
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
       <c r="B4" s="4" t="str">
-        <f>IF(A4="","",CHOOSE(WEEKDAY(A4,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <f>IF(A4="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A4),A4,DATEVALUE(A4)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
         <v/>
       </c>
       <c r="C4" s="5"/>
@@ -526,18 +524,18 @@
         <f>IF(AND(C4&lt;&gt;"",D4&lt;&gt;""),(D4-C4)*24-E4/60,"")</f>
         <v/>
       </c>
-      <c r="G4" s="8"/>
+      <c r="G4" s="4"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="9"/>
-      <c r="B5" s="10" t="str">
-        <f>IF(A5="","",CHOOSE(WEEKDAY(A5,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
-        <v/>
-      </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="13" t="str">
+      <c r="A5" s="8"/>
+      <c r="B5" t="str">
+        <f>IF(A5="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A5),A5,DATEVALUE(A5)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
+        <v/>
+      </c>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="11" t="str">
         <f>IF(AND(C5&lt;&gt;"",D5&lt;&gt;""),(D5-C5)*24-E5/60,"")</f>
         <v/>
       </c>
@@ -545,7 +543,7 @@
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
       <c r="B6" s="4" t="str">
-        <f>IF(A6="","",CHOOSE(WEEKDAY(A6,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <f>IF(A6="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A6),A6,DATEVALUE(A6)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
         <v/>
       </c>
       <c r="C6" s="5"/>
@@ -555,18 +553,18 @@
         <f>IF(AND(C6&lt;&gt;"",D6&lt;&gt;""),(D6-C6)*24-E6/60,"")</f>
         <v/>
       </c>
-      <c r="G6" s="8"/>
+      <c r="G6" s="4"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="9"/>
-      <c r="B7" s="10" t="str">
-        <f>IF(A7="","",CHOOSE(WEEKDAY(A7,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
-        <v/>
-      </c>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="13" t="str">
+      <c r="A7" s="8"/>
+      <c r="B7" t="str">
+        <f>IF(A7="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A7),A7,DATEVALUE(A7)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
+        <v/>
+      </c>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="11" t="str">
         <f>IF(AND(C7&lt;&gt;"",D7&lt;&gt;""),(D7-C7)*24-E7/60,"")</f>
         <v/>
       </c>
@@ -574,7 +572,7 @@
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
       <c r="B8" s="4" t="str">
-        <f>IF(A8="","",CHOOSE(WEEKDAY(A8,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <f>IF(A8="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A8),A8,DATEVALUE(A8)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
         <v/>
       </c>
       <c r="C8" s="5"/>
@@ -584,18 +582,18 @@
         <f>IF(AND(C8&lt;&gt;"",D8&lt;&gt;""),(D8-C8)*24-E8/60,"")</f>
         <v/>
       </c>
-      <c r="G8" s="8"/>
+      <c r="G8" s="4"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="9"/>
-      <c r="B9" s="10" t="str">
-        <f>IF(A9="","",CHOOSE(WEEKDAY(A9,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
-        <v/>
-      </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="13" t="str">
+      <c r="A9" s="8"/>
+      <c r="B9" t="str">
+        <f>IF(A9="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A9),A9,DATEVALUE(A9)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
+        <v/>
+      </c>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="11" t="str">
         <f>IF(AND(C9&lt;&gt;"",D9&lt;&gt;""),(D9-C9)*24-E9/60,"")</f>
         <v/>
       </c>
@@ -603,7 +601,7 @@
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" s="4" t="str">
-        <f>IF(A10="","",CHOOSE(WEEKDAY(A10,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <f>IF(A10="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A10),A10,DATEVALUE(A10)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
         <v/>
       </c>
       <c r="C10" s="5"/>
@@ -613,18 +611,18 @@
         <f>IF(AND(C10&lt;&gt;"",D10&lt;&gt;""),(D10-C10)*24-E10/60,"")</f>
         <v/>
       </c>
-      <c r="G10" s="8"/>
+      <c r="G10" s="4"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="9"/>
-      <c r="B11" s="10" t="str">
-        <f>IF(A11="","",CHOOSE(WEEKDAY(A11,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
-        <v/>
-      </c>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="13" t="str">
+      <c r="A11" s="8"/>
+      <c r="B11" t="str">
+        <f>IF(A11="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A11),A11,DATEVALUE(A11)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
+        <v/>
+      </c>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="11" t="str">
         <f>IF(AND(C11&lt;&gt;"",D11&lt;&gt;""),(D11-C11)*24-E11/60,"")</f>
         <v/>
       </c>
@@ -632,7 +630,7 @@
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" s="4" t="str">
-        <f>IF(A12="","",CHOOSE(WEEKDAY(A12,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <f>IF(A12="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A12),A12,DATEVALUE(A12)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
         <v/>
       </c>
       <c r="C12" s="5"/>
@@ -642,18 +640,18 @@
         <f>IF(AND(C12&lt;&gt;"",D12&lt;&gt;""),(D12-C12)*24-E12/60,"")</f>
         <v/>
       </c>
-      <c r="G12" s="8"/>
+      <c r="G12" s="4"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="9"/>
-      <c r="B13" s="10" t="str">
-        <f>IF(A13="","",CHOOSE(WEEKDAY(A13,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
-        <v/>
-      </c>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="13" t="str">
+      <c r="A13" s="8"/>
+      <c r="B13" t="str">
+        <f>IF(A13="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A13),A13,DATEVALUE(A13)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
+        <v/>
+      </c>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="11" t="str">
         <f>IF(AND(C13&lt;&gt;"",D13&lt;&gt;""),(D13-C13)*24-E13/60,"")</f>
         <v/>
       </c>
@@ -661,7 +659,7 @@
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="4" t="str">
-        <f>IF(A14="","",CHOOSE(WEEKDAY(A14,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <f>IF(A14="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A14),A14,DATEVALUE(A14)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
         <v/>
       </c>
       <c r="C14" s="5"/>
@@ -671,18 +669,18 @@
         <f>IF(AND(C14&lt;&gt;"",D14&lt;&gt;""),(D14-C14)*24-E14/60,"")</f>
         <v/>
       </c>
-      <c r="G14" s="8"/>
+      <c r="G14" s="4"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="9"/>
-      <c r="B15" s="10" t="str">
-        <f>IF(A15="","",CHOOSE(WEEKDAY(A15,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
-        <v/>
-      </c>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="13" t="str">
+      <c r="A15" s="8"/>
+      <c r="B15" t="str">
+        <f>IF(A15="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A15),A15,DATEVALUE(A15)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
+        <v/>
+      </c>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="11" t="str">
         <f>IF(AND(C15&lt;&gt;"",D15&lt;&gt;""),(D15-C15)*24-E15/60,"")</f>
         <v/>
       </c>
@@ -690,7 +688,7 @@
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="4" t="str">
-        <f>IF(A16="","",CHOOSE(WEEKDAY(A16,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <f>IF(A16="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A16),A16,DATEVALUE(A16)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
         <v/>
       </c>
       <c r="C16" s="5"/>
@@ -700,18 +698,18 @@
         <f>IF(AND(C16&lt;&gt;"",D16&lt;&gt;""),(D16-C16)*24-E16/60,"")</f>
         <v/>
       </c>
-      <c r="G16" s="8"/>
+      <c r="G16" s="4"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="9"/>
-      <c r="B17" s="10" t="str">
-        <f>IF(A17="","",CHOOSE(WEEKDAY(A17,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
-        <v/>
-      </c>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="13" t="str">
+      <c r="A17" s="8"/>
+      <c r="B17" t="str">
+        <f>IF(A17="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A17),A17,DATEVALUE(A17)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
+        <v/>
+      </c>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="11" t="str">
         <f>IF(AND(C17&lt;&gt;"",D17&lt;&gt;""),(D17-C17)*24-E17/60,"")</f>
         <v/>
       </c>
@@ -719,7 +717,7 @@
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
       <c r="B18" s="4" t="str">
-        <f>IF(A18="","",CHOOSE(WEEKDAY(A18,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <f>IF(A18="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A18),A18,DATEVALUE(A18)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
         <v/>
       </c>
       <c r="C18" s="5"/>
@@ -729,18 +727,18 @@
         <f>IF(AND(C18&lt;&gt;"",D18&lt;&gt;""),(D18-C18)*24-E18/60,"")</f>
         <v/>
       </c>
-      <c r="G18" s="8"/>
+      <c r="G18" s="4"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="9"/>
-      <c r="B19" s="10" t="str">
-        <f>IF(A19="","",CHOOSE(WEEKDAY(A19,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
-        <v/>
-      </c>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="13" t="str">
+      <c r="A19" s="8"/>
+      <c r="B19" t="str">
+        <f>IF(A19="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A19),A19,DATEVALUE(A19)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
+        <v/>
+      </c>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="11" t="str">
         <f>IF(AND(C19&lt;&gt;"",D19&lt;&gt;""),(D19-C19)*24-E19/60,"")</f>
         <v/>
       </c>
@@ -748,7 +746,7 @@
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="4" t="str">
-        <f>IF(A20="","",CHOOSE(WEEKDAY(A20,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <f>IF(A20="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A20),A20,DATEVALUE(A20)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
         <v/>
       </c>
       <c r="C20" s="5"/>
@@ -758,18 +756,18 @@
         <f>IF(AND(C20&lt;&gt;"",D20&lt;&gt;""),(D20-C20)*24-E20/60,"")</f>
         <v/>
       </c>
-      <c r="G20" s="8"/>
+      <c r="G20" s="4"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="9"/>
-      <c r="B21" s="10" t="str">
-        <f>IF(A21="","",CHOOSE(WEEKDAY(A21,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
-        <v/>
-      </c>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="13" t="str">
+      <c r="A21" s="8"/>
+      <c r="B21" t="str">
+        <f>IF(A21="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A21),A21,DATEVALUE(A21)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
+        <v/>
+      </c>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="11" t="str">
         <f>IF(AND(C21&lt;&gt;"",D21&lt;&gt;""),(D21-C21)*24-E21/60,"")</f>
         <v/>
       </c>
@@ -777,7 +775,7 @@
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
       <c r="B22" s="4" t="str">
-        <f>IF(A22="","",CHOOSE(WEEKDAY(A22,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <f>IF(A22="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A22),A22,DATEVALUE(A22)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
         <v/>
       </c>
       <c r="C22" s="5"/>
@@ -787,18 +785,18 @@
         <f>IF(AND(C22&lt;&gt;"",D22&lt;&gt;""),(D22-C22)*24-E22/60,"")</f>
         <v/>
       </c>
-      <c r="G22" s="8"/>
+      <c r="G22" s="4"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="9"/>
-      <c r="B23" s="10" t="str">
-        <f>IF(A23="","",CHOOSE(WEEKDAY(A23,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
-        <v/>
-      </c>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="12"/>
-      <c r="F23" s="13" t="str">
+      <c r="A23" s="8"/>
+      <c r="B23" t="str">
+        <f>IF(A23="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A23),A23,DATEVALUE(A23)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
+        <v/>
+      </c>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="11" t="str">
         <f>IF(AND(C23&lt;&gt;"",D23&lt;&gt;""),(D23-C23)*24-E23/60,"")</f>
         <v/>
       </c>
@@ -806,7 +804,7 @@
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" s="4" t="str">
-        <f>IF(A24="","",CHOOSE(WEEKDAY(A24,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <f>IF(A24="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A24),A24,DATEVALUE(A24)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
         <v/>
       </c>
       <c r="C24" s="5"/>
@@ -816,18 +814,18 @@
         <f>IF(AND(C24&lt;&gt;"",D24&lt;&gt;""),(D24-C24)*24-E24/60,"")</f>
         <v/>
       </c>
-      <c r="G24" s="8"/>
+      <c r="G24" s="4"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="9"/>
-      <c r="B25" s="10" t="str">
-        <f>IF(A25="","",CHOOSE(WEEKDAY(A25,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
-        <v/>
-      </c>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="13" t="str">
+      <c r="A25" s="8"/>
+      <c r="B25" t="str">
+        <f>IF(A25="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A25),A25,DATEVALUE(A25)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
+        <v/>
+      </c>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="11" t="str">
         <f>IF(AND(C25&lt;&gt;"",D25&lt;&gt;""),(D25-C25)*24-E25/60,"")</f>
         <v/>
       </c>
@@ -835,7 +833,7 @@
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
       <c r="B26" s="4" t="str">
-        <f>IF(A26="","",CHOOSE(WEEKDAY(A26,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <f>IF(A26="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A26),A26,DATEVALUE(A26)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
         <v/>
       </c>
       <c r="C26" s="5"/>
@@ -845,18 +843,18 @@
         <f>IF(AND(C26&lt;&gt;"",D26&lt;&gt;""),(D26-C26)*24-E26/60,"")</f>
         <v/>
       </c>
-      <c r="G26" s="8"/>
+      <c r="G26" s="4"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="9"/>
-      <c r="B27" s="10" t="str">
-        <f>IF(A27="","",CHOOSE(WEEKDAY(A27,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
-        <v/>
-      </c>
-      <c r="C27" s="11"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="12"/>
-      <c r="F27" s="13" t="str">
+      <c r="A27" s="8"/>
+      <c r="B27" t="str">
+        <f>IF(A27="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A27),A27,DATEVALUE(A27)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
+        <v/>
+      </c>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="11" t="str">
         <f>IF(AND(C27&lt;&gt;"",D27&lt;&gt;""),(D27-C27)*24-E27/60,"")</f>
         <v/>
       </c>
@@ -864,7 +862,7 @@
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="B28" s="4" t="str">
-        <f>IF(A28="","",CHOOSE(WEEKDAY(A28,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <f>IF(A28="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A28),A28,DATEVALUE(A28)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
         <v/>
       </c>
       <c r="C28" s="5"/>
@@ -874,18 +872,18 @@
         <f>IF(AND(C28&lt;&gt;"",D28&lt;&gt;""),(D28-C28)*24-E28/60,"")</f>
         <v/>
       </c>
-      <c r="G28" s="8"/>
+      <c r="G28" s="4"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="9"/>
-      <c r="B29" s="10" t="str">
-        <f>IF(A29="","",CHOOSE(WEEKDAY(A29,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
-        <v/>
-      </c>
-      <c r="C29" s="11"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="12"/>
-      <c r="F29" s="13" t="str">
+      <c r="A29" s="8"/>
+      <c r="B29" t="str">
+        <f>IF(A29="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A29),A29,DATEVALUE(A29)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
+        <v/>
+      </c>
+      <c r="C29" s="9"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="11" t="str">
         <f>IF(AND(C29&lt;&gt;"",D29&lt;&gt;""),(D29-C29)*24-E29/60,"")</f>
         <v/>
       </c>
@@ -893,7 +891,7 @@
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="4" t="str">
-        <f>IF(A30="","",CHOOSE(WEEKDAY(A30,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <f>IF(A30="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A30),A30,DATEVALUE(A30)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
         <v/>
       </c>
       <c r="C30" s="5"/>
@@ -903,18 +901,18 @@
         <f>IF(AND(C30&lt;&gt;"",D30&lt;&gt;""),(D30-C30)*24-E30/60,"")</f>
         <v/>
       </c>
-      <c r="G30" s="8"/>
+      <c r="G30" s="4"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="9"/>
-      <c r="B31" s="10" t="str">
-        <f>IF(A31="","",CHOOSE(WEEKDAY(A31,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
-        <v/>
-      </c>
-      <c r="C31" s="11"/>
-      <c r="D31" s="11"/>
-      <c r="E31" s="12"/>
-      <c r="F31" s="13" t="str">
+      <c r="A31" s="8"/>
+      <c r="B31" t="str">
+        <f>IF(A31="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A31),A31,DATEVALUE(A31)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
+        <v/>
+      </c>
+      <c r="C31" s="9"/>
+      <c r="D31" s="9"/>
+      <c r="E31" s="10"/>
+      <c r="F31" s="11" t="str">
         <f>IF(AND(C31&lt;&gt;"",D31&lt;&gt;""),(D31-C31)*24-E31/60,"")</f>
         <v/>
       </c>
@@ -922,7 +920,7 @@
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="4" t="str">
-        <f>IF(A32="","",CHOOSE(WEEKDAY(A32,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
+        <f>IF(A32="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A32),A32,DATEVALUE(A32)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
         <v/>
       </c>
       <c r="C32" s="5"/>
@@ -932,27 +930,27 @@
         <f>IF(AND(C32&lt;&gt;"",D32&lt;&gt;""),(D32-C32)*24-E32/60,"")</f>
         <v/>
       </c>
-      <c r="G32" s="8"/>
+      <c r="G32" s="4"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="9"/>
-      <c r="B33" s="10" t="str">
-        <f>IF(A33="","",CHOOSE(WEEKDAY(A33,2),"ponedeljek","torek","sreda","četrtek","petek","sobota","nedelja"))</f>
-        <v/>
-      </c>
-      <c r="C33" s="11"/>
-      <c r="D33" s="11"/>
-      <c r="E33" s="12"/>
-      <c r="F33" s="13" t="str">
+      <c r="A33" s="8"/>
+      <c r="B33" t="str">
+        <f>IF(A33="","",IFERROR(CHOOSE(WEEKDAY(IF(ISNUMBER(A33),A33,DATEVALUE(A33)),2),"Ponedeljek","Torek","Sreda","Četrtek","Petek","Sobota","Nedelja"),""))</f>
+        <v/>
+      </c>
+      <c r="C33" s="9"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="11" t="str">
         <f>IF(AND(C33&lt;&gt;"",D33&lt;&gt;""),(D33-C33)*24-E33/60,"")</f>
         <v/>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="14" t="s">
+      <c r="A35" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="F35" s="15">
+      <c r="F35" s="13">
         <f>SUM(F2:F33)</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Excel sample: add usage instructions (date format) below the table
Add a "Navodilo za uporabo" block under the table explaining the date
format (dd.mm.llll), time entry and a PDF-export tip, plus a cell comment
on the Datum header. Helps users enter dates so the weekday/total compute.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/vzorec-evidenca-delovnega-casa.xlsx
+++ b/public/vzorec-evidenca-delovnega-casa.xlsx
@@ -10,8 +10,25 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0">
+      <text>
+        <r>
+          <t>Datum vpišite kot dd.mm.llll (npr. 03.07.2026). Dan v tednu se izpiše samodejno.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Datum</t>
   </si>
@@ -35,6 +52,21 @@
   </si>
   <si>
     <t>SKUPAJ</t>
+  </si>
+  <si>
+    <t>Navodilo za uporabo</t>
+  </si>
+  <si>
+    <t>Datum vpišite v obliki dd.mm.llll, npr. 03.07.2026. Dan v tednu in »Skupaj ur« se izračunata samodejno.</t>
+  </si>
+  <si>
+    <t>Prihod in odhod vpišite kot uro, npr. 08:00 in 16:00. Odmor vpišite v minutah (npr. 30).</t>
+  </si>
+  <si>
+    <t>Nasvet: ob koncu meseca datoteko shranite ali izvozite v PDF (nespremenljiva oblika za inšpekcijo).</t>
+  </si>
+  <si>
+    <t>Pripravljeno z Delovit · www.delovit.si</t>
   </si>
 </sst>
 </file>
@@ -45,7 +77,7 @@
     <numFmt numFmtId="164" formatCode="dd.mm.yyyy"/>
     <numFmt numFmtId="165" formatCode="hh:mm"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -60,6 +92,15 @@
     </font>
     <font>
       <b/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF1D4ED8"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="FF475569"/>
+      <sz val="10.5"/>
     </font>
   </fonts>
   <fills count="4">
@@ -92,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -111,6 +152,12 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -450,7 +497,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -955,8 +1002,71 @@
         <v>0</v>
       </c>
     </row>
+    <row r="38" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B38" s="14"/>
+      <c r="C38" s="14"/>
+      <c r="D38" s="14"/>
+      <c r="E38" s="14"/>
+      <c r="F38" s="14"/>
+      <c r="G38" s="14"/>
+    </row>
+    <row r="39" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="B39" s="15"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="15"/>
+      <c r="E39" s="15"/>
+      <c r="F39" s="15"/>
+      <c r="G39" s="15"/>
+    </row>
+    <row r="40" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B40" s="15"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="15"/>
+      <c r="E40" s="15"/>
+      <c r="F40" s="15"/>
+      <c r="G40" s="15"/>
+    </row>
+    <row r="41" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B41" s="15"/>
+      <c r="C41" s="15"/>
+      <c r="D41" s="15"/>
+      <c r="E41" s="15"/>
+      <c r="F41" s="15"/>
+      <c r="G41" s="15"/>
+    </row>
+    <row r="42" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B42" s="15"/>
+      <c r="C42" s="15"/>
+      <c r="D42" s="15"/>
+      <c r="E42" s="15"/>
+      <c r="F42" s="15"/>
+      <c r="G42" s="15"/>
+    </row>
   </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A38:G38"/>
+    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="A41:G41"/>
+    <mergeCell ref="A42:G42"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Excel sample: clarify date format note (dots vs slashes by locale)
The instruction now covers both cases: dd.mm.llll (e.g. 3.5.2026) for
Slovenian/Sheets, and a fallback line to use slashes (3/5/2026) if Excel
with non-Slovenian regional settings doesn't show the weekday. Cell comment
on Datum updated to match.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/vzorec-evidenca-delovnega-casa.xlsx
+++ b/public/vzorec-evidenca-delovnega-casa.xlsx
@@ -19,7 +19,7 @@
     <comment ref="A1" authorId="0">
       <text>
         <r>
-          <t>Datum vpišite kot dd.mm.llll (npr. 03.07.2026). Dan v tednu se izpiše samodejno.</t>
+          <t>Datum vpišite kot 3.5.2026. Če se v Excelu »Dan v tednu« ne izpiše, vpišite datum s poševnico: 3/5/2026.</t>
         </r>
       </text>
     </comment>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Datum</t>
   </si>
@@ -57,13 +57,16 @@
     <t>Navodilo za uporabo</t>
   </si>
   <si>
-    <t>Datum vpišite v obliki dd.mm.llll, npr. 03.07.2026. Dan v tednu in »Skupaj ur« se izračunata samodejno.</t>
-  </si>
-  <si>
-    <t>Prihod in odhod vpišite kot uro, npr. 08:00 in 16:00. Odmor vpišite v minutah (npr. 30).</t>
-  </si>
-  <si>
-    <t>Nasvet: ob koncu meseca datoteko shranite ali izvozite v PDF (nespremenljiva oblika za inšpekcijo).</t>
+    <t>Datum vpišite kot 3.5.2026 (dan.mesec.leto). Dan v tednu in »Skupaj ur« se izračunata samodejno.</t>
+  </si>
+  <si>
+    <t>Če uporabljate Excel z neslovenskimi nastavitvami in se »Dan v tednu« ne izpiše, vpišite datum s poševnico: 3/5/2026.</t>
+  </si>
+  <si>
+    <t>Prihod in odhod vpišite kot uro (npr. 08:00 in 16:00), odmor v minutah (npr. 30).</t>
+  </si>
+  <si>
+    <t>Nasvet: ob koncu meseca datoteko izvozite v PDF (nespremenljiva oblika za inšpekcijo).</t>
   </si>
   <si>
     <t>Pripravljeno z Delovit · www.delovit.si</t>
@@ -497,7 +500,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -1057,13 +1060,25 @@
       <c r="F42" s="15"/>
       <c r="G42" s="15"/>
     </row>
+    <row r="43" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B43" s="15"/>
+      <c r="C43" s="15"/>
+      <c r="D43" s="15"/>
+      <c r="E43" s="15"/>
+      <c r="F43" s="15"/>
+      <c r="G43" s="15"/>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A38:G38"/>
     <mergeCell ref="A39:G39"/>
     <mergeCell ref="A40:G40"/>
     <mergeCell ref="A41:G41"/>
     <mergeCell ref="A42:G42"/>
+    <mergeCell ref="A43:G43"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>